<commit_message>
refactor: simplify Request model and cleanup schema inconsistencies
- Removed nested RequestEnvelope abstraction
- Flattened Request.cs to align with request-schema.v1.json
- Adjusted deserialization logic in RequestDeserializer
- Removed unused properties and fixed BC30456 errors
- Adapted test inputs and Process.xaml to match new structure
</commit_message>
<xml_diff>
--- a/contentFiles/any/any/pt2/VisualBasic/Data/Testdata/Scratch.xlsx
+++ b/contentFiles/any/any/pt2/VisualBasic/Data/Testdata/Scratch.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github.com\rpapub\MaestroTaskProcess\contentFiles\any\any\pt2\VisualBasic\Data\Testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DBB2352-2019-4268-A0CF-F79E7D22EFB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8FA6290-73B9-4C71-90E9-74117EB52580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1590" yWindow="4230" windowWidth="28800" windowHeight="17685" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-2910" yWindow="10260" windowWidth="28800" windowHeight="17685" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="35">
   <si>
     <t>v1</t>
   </si>
@@ -39,12 +39,6 @@
     <t>2025-07-06T10:30:00Z</t>
   </si>
   <si>
-    <t>DataImport</t>
-  </si>
-  <si>
-    <t>trigger-snapshot</t>
-  </si>
-  <si>
     <t>223e4567-e89b-12d3-a456-426614174111</t>
   </si>
   <si>
@@ -54,12 +48,6 @@
     <t>2025-07-06T10:45:00Z</t>
   </si>
   <si>
-    <t>InvoiceProcessor</t>
-  </si>
-  <si>
-    <t>start-invoice-processing</t>
-  </si>
-  <si>
     <t>323e4567-e89b-12d3-a456-426614174222</t>
   </si>
   <si>
@@ -69,12 +57,6 @@
     <t>2025-07-06T11:00:00Z</t>
   </si>
   <si>
-    <t>CustomerCleanup</t>
-  </si>
-  <si>
-    <t>cleanup-orphan-records</t>
-  </si>
-  <si>
     <t>in_IsSuccessExpected</t>
   </si>
   <si>
@@ -103,13 +85,58 @@
   </si>
   <si>
     <t>dev</t>
+  </si>
+  <si>
+    <t>req-004</t>
+  </si>
+  <si>
+    <t>req-005</t>
+  </si>
+  <si>
+    <t>123e4567-e89b-12d3-a456-426614174333</t>
+  </si>
+  <si>
+    <t>223e4567-e89b-12d3-a456-426614174444</t>
+  </si>
+  <si>
+    <t>2025-07-06T11:15:00Z</t>
+  </si>
+  <si>
+    <t>2025-07-06T11:30:00Z</t>
+  </si>
+  <si>
+    <t>BRE</t>
+  </si>
+  <si>
+    <t>retryable</t>
+  </si>
+  <si>
+    <t>nonRetryable</t>
+  </si>
+  <si>
+    <t>timeout</t>
+  </si>
+  <si>
+    <t>sysex</t>
+  </si>
+  <si>
+    <t>foo</t>
+  </si>
+  <si>
+    <t>223e4567-e89b-12d3-a456-426614174555</t>
+  </si>
+  <si>
+    <t>req-006</t>
+  </si>
+  <si>
+    <t>2025-07-06T11:45:00Z</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -121,6 +148,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -430,7 +463,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
@@ -439,43 +472,43 @@
     <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="34.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>24</v>
-      </c>
       <c r="H1" s="2" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
@@ -489,69 +522,130 @@
       <c r="E2" t="s">
         <v>3</v>
       </c>
-      <c r="F2" t="s">
-        <v>4</v>
-      </c>
       <c r="G2" t="s">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="H2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" t="s">
         <v>6</v>
       </c>
-      <c r="D3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
       <c r="G3" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="H3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" t="s">
         <v>25</v>
       </c>
-      <c r="B4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" t="b">
+      <c r="G6" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7" t="s">
+        <v>31</v>
+      </c>
+      <c r="H7" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>